<commit_message>
whatsap email volunteer headerfooter module fixes
</commit_message>
<xml_diff>
--- a/seva-frontend/public/sample_broadcast_contacts.xlsx
+++ b/seva-frontend/public/sample_broadcast_contacts.xlsx
@@ -397,57 +397,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Name</v>
       </c>
       <c r="B1" t="str">
-        <v>Phone</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Campaign</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Email</v>
+        <v>Mobile Number</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Rajesh Sharma</v>
+        <v>Saksham Sharma</v>
       </c>
       <c r="B2" t="str">
-        <v>9876543210</v>
-      </c>
-      <c r="C2" t="str">
-        <v>1000</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Clean Water Initiative</v>
-      </c>
-      <c r="E2" t="str">
-        <v>rajesh@example.com</v>
+        <v>+919876543210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Pooja Verma</v>
+        <v>Priya Verma</v>
       </c>
       <c r="B3" t="str">
-        <v>9123456780</v>
-      </c>
-      <c r="C3" t="str">
-        <v>2500</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Girl Child Education</v>
-      </c>
-      <c r="E3" t="str">
-        <v>pooja@example.com</v>
+        <v>+919123456789</v>
       </c>
     </row>
     <row r="4">
@@ -455,38 +432,20 @@
         <v>Amitabh Sen</v>
       </c>
       <c r="B4" t="str">
-        <v>9988776655</v>
-      </c>
-      <c r="C4" t="str">
-        <v>5000</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Kerala Relief Fund</v>
-      </c>
-      <c r="E4" t="str">
-        <v>amitabh@example.com</v>
+        <v>+919988776655</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Sneha Patel</v>
+        <v>Rohan Gupta</v>
       </c>
       <c r="B5" t="str">
         <v>9811223344</v>
-      </c>
-      <c r="C5" t="str">
-        <v>1500</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Healthcare Mission</v>
-      </c>
-      <c r="E5" t="str">
-        <v>sneha@example.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>